<commit_message>
20260513 : 점 하나 추가
</commit_message>
<xml_diff>
--- a/Python_2026/AnD_KPI_2026.xlsx
+++ b/Python_2026/AnD_KPI_2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\_Development_2026\Python_2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C6251F0-80C2-469D-8712-D29A885AAACA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38FC4A28-244A-43AE-841C-78FA7C12F4A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{53B19080-9F04-48C2-B8B2-0D660C2AD9E9}"/>
+    <workbookView xWindow="2145" yWindow="600" windowWidth="25725" windowHeight="14235" xr2:uid="{53B19080-9F04-48C2-B8B2-0D660C2AD9E9}"/>
   </bookViews>
   <sheets>
     <sheet name="export" sheetId="1" r:id="rId1"/>
@@ -62,9 +62,6 @@
     <t>Apr(Count)</t>
   </si>
   <si>
-    <t>tickets</t>
-  </si>
-  <si>
     <t>Very High</t>
   </si>
   <si>
@@ -221,6 +218,10 @@
   </si>
   <si>
     <t>Total</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>Meeting target date of tasks in Jira tickets</t>
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
 </sst>
@@ -841,7 +842,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -869,6 +870,9 @@
     <xf numFmtId="9" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -876,7 +880,7 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="43">
@@ -1145,16 +1149,16 @@
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="13"/>
                 <c:pt idx="1">
-                  <c:v>0.12941176470588237</c:v>
+                  <c:v>0.13414634146341464</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.24705882352941178</c:v>
+                  <c:v>0.25609756097560976</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.27058823529411763</c:v>
+                  <c:v>0.28048780487804881</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.18823529411764706</c:v>
+                  <c:v>0.1951219512195122</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1720,7 +1724,7 @@
               <c:strCache>
                 <c:ptCount val="8"/>
                 <c:pt idx="0">
-                  <c:v>tickets</c:v>
+                  <c:v>Meeting target date of tasks in Jira tickets</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>Job Status update
@@ -1879,7 +1883,7 @@
               <c:strCache>
                 <c:ptCount val="8"/>
                 <c:pt idx="0">
-                  <c:v>tickets</c:v>
+                  <c:v>Meeting target date of tasks in Jira tickets</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>Job Status update
@@ -2038,7 +2042,7 @@
               <c:strCache>
                 <c:ptCount val="8"/>
                 <c:pt idx="0">
-                  <c:v>tickets</c:v>
+                  <c:v>Meeting target date of tasks in Jira tickets</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>Job Status update
@@ -2197,7 +2201,7 @@
               <c:strCache>
                 <c:ptCount val="8"/>
                 <c:pt idx="0">
-                  <c:v>tickets</c:v>
+                  <c:v>Meeting target date of tasks in Jira tickets</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>Job Status update
@@ -3987,63 +3991,63 @@
         <v>5</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="N1" s="1" t="s">
         <v>5</v>
       </c>
       <c r="O1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="P1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>27</v>
-      </c>
-      <c r="Q1" s="1" t="s">
-        <v>28</v>
       </c>
       <c r="R1" s="1" t="s">
         <v>5</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="T1" s="1" t="s">
         <v>5</v>
       </c>
       <c r="U1" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="V1" s="1" t="s">
         <v>5</v>
       </c>
       <c r="W1" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="X1" s="1" t="s">
         <v>5</v>
       </c>
       <c r="Y1" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="Z1" s="1" t="s">
         <v>5</v>
       </c>
       <c r="AA1" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="AB1" s="1" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:28" ht="99" x14ac:dyDescent="0.3">
-      <c r="A2" s="7" t="s">
+      <c r="A2" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="B2" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="C2" s="9" t="s">
         <v>10</v>
-      </c>
-      <c r="C2" s="11" t="s">
-        <v>11</v>
       </c>
       <c r="D2" s="7">
         <v>2.5</v>
@@ -4074,14 +4078,14 @@
       </c>
     </row>
     <row r="3" spans="1:28" ht="82.5" x14ac:dyDescent="0.3">
-      <c r="A3" s="5" t="s">
+      <c r="A3" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="C3" s="9" t="s">
         <v>13</v>
-      </c>
-      <c r="C3" s="11" t="s">
-        <v>14</v>
       </c>
       <c r="D3" s="7">
         <v>2</v>
@@ -4112,14 +4116,14 @@
       </c>
     </row>
     <row r="4" spans="1:28" ht="82.5" x14ac:dyDescent="0.3">
-      <c r="A4" s="7" t="s">
-        <v>15</v>
+      <c r="A4" s="12" t="s">
+        <v>14</v>
       </c>
       <c r="B4" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" s="9" t="s">
         <v>13</v>
-      </c>
-      <c r="C4" s="11" t="s">
-        <v>14</v>
       </c>
       <c r="D4" s="7">
         <v>2</v>
@@ -4150,14 +4154,14 @@
       </c>
     </row>
     <row r="5" spans="1:28" ht="82.5" x14ac:dyDescent="0.3">
-      <c r="A5" s="5" t="s">
-        <v>16</v>
+      <c r="A5" s="9" t="s">
+        <v>15</v>
       </c>
       <c r="B5" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" s="9" t="s">
         <v>13</v>
-      </c>
-      <c r="C5" s="11" t="s">
-        <v>14</v>
       </c>
       <c r="D5" s="7">
         <v>2</v>
@@ -4188,14 +4192,14 @@
       </c>
     </row>
     <row r="6" spans="1:28" ht="66" x14ac:dyDescent="0.3">
-      <c r="A6" s="7" t="s">
+      <c r="A6" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="B6" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="C6" s="9" t="s">
         <v>18</v>
-      </c>
-      <c r="C6" s="11" t="s">
-        <v>19</v>
       </c>
       <c r="D6" s="7">
         <v>1.5</v>
@@ -4226,14 +4230,14 @@
       </c>
     </row>
     <row r="7" spans="1:28" ht="82.5" x14ac:dyDescent="0.3">
-      <c r="A7" s="5" t="s">
+      <c r="A7" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="C7" s="9" t="s">
         <v>20</v>
-      </c>
-      <c r="B7" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="C7" s="11" t="s">
-        <v>21</v>
       </c>
       <c r="D7" s="7">
         <v>2</v>
@@ -4264,14 +4268,14 @@
       </c>
     </row>
     <row r="8" spans="1:28" ht="82.5" x14ac:dyDescent="0.3">
-      <c r="A8" s="7" t="s">
-        <v>22</v>
+      <c r="A8" s="12" t="s">
+        <v>21</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="C8" s="11" t="s">
-        <v>21</v>
+        <v>12</v>
+      </c>
+      <c r="C8" s="9" t="s">
+        <v>20</v>
       </c>
       <c r="D8" s="7">
         <v>2</v>
@@ -4302,14 +4306,14 @@
       </c>
     </row>
     <row r="9" spans="1:28" ht="115.5" x14ac:dyDescent="0.3">
-      <c r="A9" s="7" t="s">
+      <c r="A9" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="C9" s="9" t="s">
         <v>23</v>
-      </c>
-      <c r="B9" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="C9" s="11" t="s">
-        <v>24</v>
       </c>
       <c r="D9" s="7">
         <v>2.5</v>
@@ -4342,10 +4346,10 @@
     <row r="10" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A10" s="7"/>
       <c r="B10" s="7" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C10" s="7">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="D10" s="5">
         <v>16.5</v>
@@ -4386,7 +4390,7 @@
       <c r="D11" s="8"/>
       <c r="E11" s="6">
         <f>(E10/$C$10)</f>
-        <v>0.12941176470588237</v>
+        <v>0.13414634146341464</v>
       </c>
       <c r="F11" s="6">
         <f>1-(F10/$D$10)</f>
@@ -4394,7 +4398,7 @@
       </c>
       <c r="G11" s="6">
         <f>(G10/$C$10)</f>
-        <v>0.24705882352941178</v>
+        <v>0.25609756097560976</v>
       </c>
       <c r="H11" s="6">
         <f>1-(H10/$D$10)</f>
@@ -4402,7 +4406,7 @@
       </c>
       <c r="I11" s="6">
         <f>(I10/$C$10)</f>
-        <v>0.27058823529411763</v>
+        <v>0.28048780487804881</v>
       </c>
       <c r="J11" s="6">
         <f>1-(J10/$D$10)</f>
@@ -4410,7 +4414,7 @@
       </c>
       <c r="K11" s="6">
         <f>(K10/$C$10)</f>
-        <v>0.18823529411764706</v>
+        <v>0.1951219512195122</v>
       </c>
       <c r="L11" s="6">
         <f>1-(L10/$D$10)</f>
@@ -4418,70 +4422,70 @@
       </c>
     </row>
     <row r="13" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="C13" s="9" t="s">
+      <c r="C13" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="D13" s="9"/>
+      <c r="D13" s="10"/>
       <c r="E13" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="F13" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="F13" s="4" t="s">
+      <c r="G13" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="G13" s="4" t="s">
+      <c r="H13" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="H13" s="4" t="s">
+      <c r="I13" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="I13" s="4" t="s">
+      <c r="J13" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="J13" s="4" t="s">
+      <c r="K13" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="K13" s="4" t="s">
+      <c r="L13" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="L13" s="4" t="s">
+      <c r="M13" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="M13" s="4" t="s">
+      <c r="N13" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="N13" s="4" t="s">
+      <c r="O13" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="O13" s="4" t="s">
+      <c r="P13" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="P13" s="4" t="s">
-        <v>46</v>
-      </c>
       <c r="Q13" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="14" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="C14" s="10" t="s">
-        <v>47</v>
-      </c>
-      <c r="D14" s="10"/>
+      <c r="C14" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="D14" s="11"/>
       <c r="E14" s="6">
         <f>(E10/$C$10)</f>
-        <v>0.12941176470588237</v>
+        <v>0.13414634146341464</v>
       </c>
       <c r="F14" s="6">
         <f>(G10/$C$10)</f>
-        <v>0.24705882352941178</v>
+        <v>0.25609756097560976</v>
       </c>
       <c r="G14" s="6">
         <f>(I10/$C$10)</f>
-        <v>0.27058823529411763</v>
+        <v>0.28048780487804881</v>
       </c>
       <c r="H14" s="6">
         <f>(K10/$C$10)</f>
-        <v>0.18823529411764706</v>
+        <v>0.1951219512195122</v>
       </c>
       <c r="I14" s="6"/>
       <c r="J14" s="6"/>
@@ -4493,14 +4497,14 @@
       <c r="P14" s="5"/>
       <c r="Q14" s="3">
         <f>AVERAGE(E14:P14)</f>
-        <v>0.20882352941176469</v>
+        <v>0.21646341463414637</v>
       </c>
     </row>
     <row r="15" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="C15" s="10" t="s">
-        <v>48</v>
-      </c>
-      <c r="D15" s="10"/>
+      <c r="C15" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="D15" s="11"/>
       <c r="E15" s="6">
         <f>1-(F10/$D$10)</f>
         <v>0.81818181818181812</v>

</xml_diff>